<commit_message>
new requests for plots
</commit_message>
<xml_diff>
--- a/docs/LC_Prominence_selection.xlsx
+++ b/docs/LC_Prominence_selection.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\My Drive\from 2018 fall\MeilingDATA\LC_GCaMP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67659711-AB28-44A4-9F52-3DA0595DE65B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E6141F69-E692-4017-A1DD-CC093FA8CA8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,24 +36,15 @@
     <t>scn1a_NOseizure</t>
   </si>
   <si>
-    <t>prominence</t>
-  </si>
-  <si>
     <t>0.025, can try lower 0.02?</t>
   </si>
   <si>
     <t>note</t>
   </si>
   <si>
-    <t>trim the first 1 min baseline data</t>
-  </si>
-  <si>
     <t>exclude the data</t>
   </si>
   <si>
-    <t>exclude the data?</t>
-  </si>
-  <si>
     <t xml:space="preserve"> can try lower 0.02?</t>
   </si>
   <si>
@@ -67,13 +58,22 @@
   </si>
   <si>
     <t>heating session #</t>
+  </si>
+  <si>
+    <t>trim the first 100s for all data</t>
+  </si>
+  <si>
+    <t>prominence (20260430)</t>
+  </si>
+  <si>
+    <t>prominence (20260427)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -84,6 +84,20 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="2" tint="-9.9978637043366805E-2"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -149,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
@@ -168,6 +182,13 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -448,38 +469,41 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="26.140625" customWidth="1"/>
     <col min="2" max="2" width="36.28515625" customWidth="1"/>
     <col min="3" max="3" width="13.28515625" customWidth="1"/>
     <col min="4" max="4" width="15.85546875" customWidth="1"/>
-    <col min="5" max="5" width="27.140625" customWidth="1"/>
-    <col min="6" max="6" width="35.42578125" customWidth="1"/>
+    <col min="5" max="6" width="27.140625" customWidth="1"/>
+    <col min="7" max="7" width="35.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="47.25" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" ht="31.5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="C1" s="3" t="s">
+      <c r="E1" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="5" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="G1" s="5" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
@@ -492,12 +516,15 @@
       <c r="D2" s="2">
         <v>1</v>
       </c>
-      <c r="E2" s="6">
+      <c r="E2" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F2" s="7"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F2" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G2" s="7"/>
+    </row>
+    <row r="3" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>0</v>
       </c>
@@ -510,12 +537,15 @@
       <c r="D3" s="1">
         <v>1</v>
       </c>
-      <c r="E3" s="6">
+      <c r="E3" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F3" s="7"/>
-    </row>
-    <row r="4" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F3" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G3" s="7"/>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>0</v>
       </c>
@@ -528,12 +558,15 @@
       <c r="D4" s="1">
         <v>2</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F4" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G4" s="7"/>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>0</v>
       </c>
@@ -546,12 +579,15 @@
       <c r="D5" s="1">
         <v>1</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F5" s="7"/>
-    </row>
-    <row r="6" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F5" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G5" s="7"/>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>1</v>
       </c>
@@ -564,12 +600,15 @@
       <c r="D6" s="1">
         <v>1</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F6" s="7"/>
-    </row>
-    <row r="7" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F6" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G6" s="7"/>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>1</v>
       </c>
@@ -582,12 +621,15 @@
       <c r="D7" s="1">
         <v>1</v>
       </c>
-      <c r="E7" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F7" s="7"/>
-    </row>
-    <row r="8" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E7" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F7" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G7" s="7"/>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>1</v>
       </c>
@@ -600,12 +642,15 @@
       <c r="D8" s="1">
         <v>1</v>
       </c>
-      <c r="E8" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F8" s="7"/>
-    </row>
-    <row r="9" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E8" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F8" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G8" s="7"/>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>1</v>
       </c>
@@ -618,12 +663,15 @@
       <c r="D9" s="1">
         <v>2</v>
       </c>
-      <c r="E9" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F9" s="7"/>
-    </row>
-    <row r="10" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E9" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F9" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G9" s="7"/>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>1</v>
       </c>
@@ -636,12 +684,15 @@
       <c r="D10" s="1">
         <v>1</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F10" s="7"/>
-    </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F10" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G10" s="7"/>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>1</v>
       </c>
@@ -654,12 +705,15 @@
       <c r="D11" s="1">
         <v>1</v>
       </c>
-      <c r="E11" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F11" s="7"/>
-    </row>
-    <row r="12" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E11" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F11" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G11" s="7"/>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>2</v>
       </c>
@@ -672,14 +726,17 @@
       <c r="D12" s="1">
         <v>1</v>
       </c>
-      <c r="E12" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F12" s="7" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E12" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F12" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G12" s="8" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>2</v>
       </c>
@@ -692,12 +749,15 @@
       <c r="D13" s="1">
         <v>2</v>
       </c>
-      <c r="E13" s="6">
+      <c r="E13" s="10">
         <v>2.5000000000000001E-2</v>
       </c>
-      <c r="F13" s="7"/>
-    </row>
-    <row r="14" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="F13" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G13" s="7"/>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>2</v>
       </c>
@@ -710,12 +770,13 @@
       <c r="D14" s="1">
         <v>1</v>
       </c>
-      <c r="E14" s="6"/>
-      <c r="F14" s="7" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E14" s="10"/>
+      <c r="F14" s="6"/>
+      <c r="G14" s="8" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>2</v>
       </c>
@@ -728,12 +789,15 @@
       <c r="D15" s="1">
         <v>1</v>
       </c>
-      <c r="E15" s="6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" s="7"/>
-    </row>
-    <row r="16" spans="1:6" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="E15" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G15" s="7"/>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>2</v>
       </c>
@@ -746,12 +810,13 @@
       <c r="D16" s="1">
         <v>1</v>
       </c>
-      <c r="E16" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="F16" s="7" t="s">
-        <v>8</v>
-      </c>
+      <c r="E16" s="10" t="s">
+        <v>3</v>
+      </c>
+      <c r="F16" s="6">
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G16" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>